<commit_message>
Enforce strict day-ahead evaluation outputs
</commit_message>
<xml_diff>
--- a/Thesis Forecasting/PAPER CONTEXT/appendix_summary.xlsx
+++ b/Thesis Forecasting/PAPER CONTEXT/appendix_summary.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Outage Legend'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Execution Commands'!$A$1:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Testing Metrics Summary'!$A$1:$K$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Picture Catalog'!$A$1:$K$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Picture Catalog'!$A$1:$K$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1555,7 +1555,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.15</v>
+        <v>0.75</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Yes (-0.005794 MW)</t>
+          <t>Yes (0.043468 MW)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>169</v>
+        <v>234</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Yes (0.002722 MW)</t>
+          <t>Yes (0.008800 MW)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2021,7 +2021,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>169</v>
+        <v>234</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Yes (0.001869 MW)</t>
+          <t>Yes (0.002246 MW)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2329,7 +2329,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.001</v>
+        <v>0.0003</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Yes (-0.013115 MW)</t>
+          <t>Yes (-0.020561 MW)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>171</v>
+        <v>276</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2667,7 +2667,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.15</v>
+        <v>0.2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2818,7 +2818,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Yes (-0.008944 MW)</t>
+          <t>Yes (-0.007211 MW)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2945,7 +2945,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.001</v>
+        <v>0.0003</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1.15</v>
+        <v>1</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Yes (0.007462 MW)</t>
+          <t>Yes (0.007701 MW)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -4168,11 +4168,11 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4244,31 +4244,31 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>158</v>
+        <v>198</v>
       </c>
       <c r="D2" t="n">
-        <v>3.471231035467674</v>
+        <v>6.153104165758873</v>
       </c>
       <c r="E2" t="n">
-        <v>1.726776719652155</v>
+        <v>2.811882025863321</v>
       </c>
       <c r="F2" t="n">
-        <v>2.755809174796953</v>
+        <v>5.479442319290094</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9290627965976143</v>
+        <v>0.6877068367595487</v>
       </c>
       <c r="H2" t="n">
-        <v>3.475919113707131</v>
+        <v>6.105778045634129</v>
       </c>
       <c r="I2" t="n">
-        <v>1.840847984937388</v>
+        <v>3.386857071797398</v>
       </c>
       <c r="J2" t="n">
-        <v>3.440295102101322</v>
+        <v>8.13895113561578</v>
       </c>
       <c r="K2" t="n">
-        <v>0.8988599585985897</v>
+        <v>0.4632597768045376</v>
       </c>
     </row>
     <row r="3">
@@ -4283,31 +4283,31 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>169</v>
+        <v>234</v>
       </c>
       <c r="D3" t="n">
-        <v>1.080237388266095</v>
+        <v>1.075889289467704</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9836404595910582</v>
+        <v>0.9788690892706671</v>
       </c>
       <c r="F3" t="n">
-        <v>4.296788174711516</v>
+        <v>4.287674615856892</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8217338979659277</v>
+        <v>0.8224893067056587</v>
       </c>
       <c r="H3" t="n">
-        <v>1.372393407127368</v>
+        <v>1.37602279744084</v>
       </c>
       <c r="I3" t="n">
-        <v>1.163875279835391</v>
+        <v>1.166965024298628</v>
       </c>
       <c r="J3" t="n">
-        <v>4.810318338249981</v>
+        <v>4.804974921892738</v>
       </c>
       <c r="K3" t="n">
-        <v>0.9120531387836908</v>
+        <v>0.9122484172061645</v>
       </c>
     </row>
     <row r="4">
@@ -4322,31 +4322,31 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>169</v>
+        <v>234</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8267609583386537</v>
+        <v>0.8175246799918215</v>
       </c>
       <c r="E4" t="n">
-        <v>0.716515938221218</v>
+        <v>0.7064718312733543</v>
       </c>
       <c r="F4" t="n">
-        <v>3.362162388246943</v>
+        <v>3.35907652459286</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9528117569485496</v>
+        <v>0.9528983379297056</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6106872916793786</v>
+        <v>0.6130007144211314</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6974508930056273</v>
+        <v>0.7005126244861353</v>
       </c>
       <c r="J4" t="n">
-        <v>3.077447039614186</v>
+        <v>3.078282641691081</v>
       </c>
       <c r="K4" t="n">
-        <v>0.9453153141242143</v>
+        <v>0.9452856136353941</v>
       </c>
     </row>
     <row r="5">
@@ -4361,31 +4361,31 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="D5" t="n">
-        <v>4.090822638647039</v>
+        <v>4.318793768964198</v>
       </c>
       <c r="E5" t="n">
-        <v>1.469152401165102</v>
+        <v>1.563576789484547</v>
       </c>
       <c r="F5" t="n">
-        <v>2.231269481513257</v>
+        <v>2.331451516613931</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9043404627666414</v>
+        <v>0.8955575617582829</v>
       </c>
       <c r="H5" t="n">
-        <v>4.039603029011061</v>
+        <v>4.096794646684014</v>
       </c>
       <c r="I5" t="n">
-        <v>1.543745650205762</v>
+        <v>1.554111766907109</v>
       </c>
       <c r="J5" t="n">
-        <v>2.189078855121269</v>
+        <v>2.26277240728757</v>
       </c>
       <c r="K5" t="n">
-        <v>0.9006571482808045</v>
+        <v>0.8938559733177291</v>
       </c>
     </row>
     <row r="6">
@@ -4400,31 +4400,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>171</v>
+        <v>276</v>
       </c>
       <c r="D6" t="n">
-        <v>2.412584472589698</v>
+        <v>2.402097920105152</v>
       </c>
       <c r="E6" t="n">
-        <v>3.667330521179721</v>
+        <v>3.650389086076817</v>
       </c>
       <c r="F6" t="n">
-        <v>7.981140072128379</v>
+        <v>7.955622016013482</v>
       </c>
       <c r="G6" t="n">
-        <v>0.83490126947832</v>
+        <v>0.835955320286343</v>
       </c>
       <c r="H6" t="n">
-        <v>1.404527208907398</v>
+        <v>1.464713478027484</v>
       </c>
       <c r="I6" t="n">
-        <v>1.395706172839505</v>
+        <v>1.421442873456793</v>
       </c>
       <c r="J6" t="n">
-        <v>5.678938424204445</v>
+        <v>5.668729123413043</v>
       </c>
       <c r="K6" t="n">
-        <v>0.9904842947984128</v>
+        <v>0.9905184777266125</v>
       </c>
     </row>
     <row r="7">
@@ -4439,31 +4439,31 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="D7" t="n">
-        <v>3.806185782809625</v>
+        <v>3.754509445274856</v>
       </c>
       <c r="E7" t="n">
-        <v>1.233536460413938</v>
+        <v>1.215632205685921</v>
       </c>
       <c r="F7" t="n">
-        <v>2.109282641716446</v>
+        <v>2.062720484862587</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8242055587670627</v>
+        <v>0.8318811757593582</v>
       </c>
       <c r="H7" t="n">
-        <v>4.209301696521237</v>
+        <v>4.223334198062059</v>
       </c>
       <c r="I7" t="n">
-        <v>1.490988678325157</v>
+        <v>1.500969941677426</v>
       </c>
       <c r="J7" t="n">
-        <v>2.254351155379669</v>
+        <v>2.224354463036969</v>
       </c>
       <c r="K7" t="n">
-        <v>0.9046698091595458</v>
+        <v>0.9071898827126064</v>
       </c>
     </row>
     <row r="8">
@@ -4478,31 +4478,31 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="D8" t="n">
-        <v>3.501692361024815</v>
+        <v>6.05848867822634</v>
       </c>
       <c r="E8" t="n">
-        <v>1.722225655240091</v>
+        <v>2.679601366339635</v>
       </c>
       <c r="F8" t="n">
-        <v>2.768729867666459</v>
+        <v>5.339435070393012</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9283960548792013</v>
+        <v>0.7034619844418862</v>
       </c>
       <c r="H8" t="n">
-        <v>3.447852956093874</v>
+        <v>6.264011727644167</v>
       </c>
       <c r="I8" t="n">
-        <v>1.839286091604038</v>
+        <v>3.465673343407024</v>
       </c>
       <c r="J8" t="n">
-        <v>3.404496657355129</v>
+        <v>8.170810627537394</v>
       </c>
       <c r="K8" t="n">
-        <v>0.9009538595396125</v>
+        <v>0.4590494702010691</v>
       </c>
     </row>
     <row r="9">
@@ -4517,31 +4517,31 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>90</v>
+        <v>229</v>
       </c>
       <c r="D9" t="n">
-        <v>2.346931442357257</v>
+        <v>8.244174327492388</v>
       </c>
       <c r="E9" t="n">
-        <v>2.305160486326509</v>
+        <v>8.262480584012122</v>
       </c>
       <c r="F9" t="n">
-        <v>4.642258055490738</v>
+        <v>12.04330344361514</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7919156409714565</v>
+        <v>-0.2911028129581079</v>
       </c>
       <c r="H9" t="n">
-        <v>2.33533295308859</v>
+        <v>12.52375367457808</v>
       </c>
       <c r="I9" t="n">
-        <v>2.09420220552992</v>
+        <v>12.86364438697415</v>
       </c>
       <c r="J9" t="n">
-        <v>5.147582401407586</v>
+        <v>18.57570150683231</v>
       </c>
       <c r="K9" t="n">
-        <v>0.8992884400653057</v>
+        <v>-0.3223620348064402</v>
       </c>
     </row>
     <row r="10">
@@ -4556,31 +4556,31 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>90</v>
+        <v>229</v>
       </c>
       <c r="D10" t="n">
-        <v>1.936903494559489</v>
+        <v>5.417944909182646</v>
       </c>
       <c r="E10" t="n">
-        <v>1.567633644343515</v>
+        <v>5.127193672709094</v>
       </c>
       <c r="F10" t="n">
-        <v>4.202708086615867</v>
+        <v>8.269477431121118</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9262681912387691</v>
+        <v>0.7108873313913491</v>
       </c>
       <c r="H10" t="n">
-        <v>2.239408662781647</v>
+        <v>6.486507480932811</v>
       </c>
       <c r="I10" t="n">
-        <v>2.837622642426907</v>
+        <v>8.186374988883136</v>
       </c>
       <c r="J10" t="n">
-        <v>4.652194045140062</v>
+        <v>10.54438607873526</v>
       </c>
       <c r="K10" t="n">
-        <v>0.8750316061125879</v>
+        <v>0.3588665486066156</v>
       </c>
     </row>
     <row r="11">
@@ -4595,31 +4595,31 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>69</v>
+        <v>208</v>
       </c>
       <c r="D11" t="n">
-        <v>4.238571959461349</v>
+        <v>10.55492248548842</v>
       </c>
       <c r="E11" t="n">
-        <v>1.516569530483253</v>
+        <v>3.379175217776207</v>
       </c>
       <c r="F11" t="n">
-        <v>2.238807395827607</v>
+        <v>5.010023433893158</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9036930363532821</v>
+        <v>0.4544590404655644</v>
       </c>
       <c r="H11" t="n">
-        <v>4.30040395222705</v>
+        <v>7.511686904047209</v>
       </c>
       <c r="I11" t="n">
-        <v>1.646964171250341</v>
+        <v>2.671366219442956</v>
       </c>
       <c r="J11" t="n">
-        <v>2.305944257556542</v>
+        <v>3.758669009569813</v>
       </c>
       <c r="K11" t="n">
-        <v>0.8897670525211819</v>
+        <v>0.7277478315778818</v>
       </c>
     </row>
     <row r="12">
@@ -4634,31 +4634,31 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>132</v>
+        <v>271</v>
       </c>
       <c r="D12" t="n">
-        <v>3.222090472477653</v>
+        <v>19.76406097356364</v>
       </c>
       <c r="E12" t="n">
-        <v>4.938827657538766</v>
+        <v>30.27459950936974</v>
       </c>
       <c r="F12" t="n">
-        <v>8.273559370524294</v>
+        <v>37.05595622095722</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8225816060696165</v>
+        <v>-2.52307734939347</v>
       </c>
       <c r="H12" t="n">
-        <v>20.54777679547323</v>
+        <v>14.82343687136343</v>
       </c>
       <c r="I12" t="n">
-        <v>9.430290892648204</v>
+        <v>16.69977506382963</v>
       </c>
       <c r="J12" t="n">
-        <v>12.42113967086908</v>
+        <v>28.36984551932682</v>
       </c>
       <c r="K12" t="n">
-        <v>0.9544771388351685</v>
+        <v>0.7613413653292103</v>
       </c>
     </row>
     <row r="13">
@@ -4673,31 +4673,31 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>69</v>
+        <v>208</v>
       </c>
       <c r="D13" t="n">
-        <v>4.158230568291292</v>
+        <v>8.358686897884775</v>
       </c>
       <c r="E13" t="n">
-        <v>1.337182294123551</v>
+        <v>2.677038225290983</v>
       </c>
       <c r="F13" t="n">
-        <v>2.071133559933018</v>
+        <v>3.814916194364496</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8305069898727634</v>
+        <v>0.4045796665847206</v>
       </c>
       <c r="H13" t="n">
-        <v>4.239258178453239</v>
+        <v>6.59874955990287</v>
       </c>
       <c r="I13" t="n">
-        <v>1.502540638105792</v>
+        <v>2.242960360791789</v>
       </c>
       <c r="J13" t="n">
-        <v>2.150702262421912</v>
+        <v>3.250476284606959</v>
       </c>
       <c r="K13" t="n">
-        <v>0.9132343321080806</v>
+        <v>0.8052767670392167</v>
       </c>
     </row>
     <row r="14">
@@ -4712,31 +4712,31 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="D14" t="n">
-        <v>3.442178031301716</v>
+        <v>12.67904447374227</v>
       </c>
       <c r="E14" t="n">
-        <v>1.707441965132599</v>
+        <v>6.199859678247157</v>
       </c>
       <c r="F14" t="n">
-        <v>2.72254522952243</v>
+        <v>9.053472191828156</v>
       </c>
       <c r="G14" t="n">
-        <v>0.9307649537783601</v>
+        <v>0.1474495234600094</v>
       </c>
       <c r="H14" t="n">
-        <v>3.509399379877545</v>
+        <v>14.89827152521508</v>
       </c>
       <c r="I14" t="n">
-        <v>1.878446300181587</v>
+        <v>8.374156805655712</v>
       </c>
       <c r="J14" t="n">
-        <v>3.476054852101562</v>
+        <v>12.32075573692778</v>
       </c>
       <c r="K14" t="n">
-        <v>0.8967464541495956</v>
+        <v>-0.2299910619096863</v>
       </c>
     </row>
     <row r="15">
@@ -4751,31 +4751,31 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>229</v>
       </c>
       <c r="D15" t="n">
-        <v>2.530532639110426</v>
+        <v>8.012625712616954</v>
       </c>
       <c r="E15" t="n">
-        <v>2.488818946565228</v>
+        <v>7.965410476549016</v>
       </c>
       <c r="F15" t="n">
-        <v>5.069029658409963</v>
+        <v>11.44105689872277</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7518978404406891</v>
+        <v>-0.1652037139806954</v>
       </c>
       <c r="H15" t="n">
-        <v>3.171957013040032</v>
+        <v>11.11757252065611</v>
       </c>
       <c r="I15" t="n">
-        <v>2.881007947430395</v>
+        <v>11.08684116555558</v>
       </c>
       <c r="J15" t="n">
-        <v>5.725848741114103</v>
+        <v>15.96858331402931</v>
       </c>
       <c r="K15" t="n">
-        <v>0.8753901278951386</v>
+        <v>0.02277920160870939</v>
       </c>
     </row>
     <row r="16">
@@ -4790,31 +4790,31 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>229</v>
       </c>
       <c r="D16" t="n">
-        <v>1.733123207504459</v>
+        <v>5.759259863862858</v>
       </c>
       <c r="E16" t="n">
-        <v>1.39760265235116</v>
+        <v>5.377330824484067</v>
       </c>
       <c r="F16" t="n">
-        <v>3.837274827912132</v>
+        <v>11.9102742084685</v>
       </c>
       <c r="G16" t="n">
-        <v>0.938532967589625</v>
+        <v>0.400271744693631</v>
       </c>
       <c r="H16" t="n">
-        <v>1.122891815055167</v>
+        <v>6.021769925483243</v>
       </c>
       <c r="I16" t="n">
-        <v>1.360446344679844</v>
+        <v>7.438204439875792</v>
       </c>
       <c r="J16" t="n">
-        <v>3.201513621959849</v>
+        <v>10.783571771579</v>
       </c>
       <c r="K16" t="n">
-        <v>0.9408172346219235</v>
+        <v>0.3294500951967373</v>
       </c>
     </row>
     <row r="17">
@@ -4829,31 +4829,31 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>69</v>
+        <v>208</v>
       </c>
       <c r="D17" t="n">
-        <v>4.228837825239769</v>
+        <v>9.792670650301922</v>
       </c>
       <c r="E17" t="n">
-        <v>1.493498170948233</v>
+        <v>3.047561809257031</v>
       </c>
       <c r="F17" t="n">
-        <v>2.204112165219101</v>
+        <v>4.714574207131379</v>
       </c>
       <c r="G17" t="n">
-        <v>0.9066548822164839</v>
+        <v>0.516904713062379</v>
       </c>
       <c r="H17" t="n">
-        <v>4.46530894611712</v>
+        <v>7.531215584620392</v>
       </c>
       <c r="I17" t="n">
-        <v>1.728274721971049</v>
+        <v>2.668592610358417</v>
       </c>
       <c r="J17" t="n">
-        <v>2.324389837729373</v>
+        <v>3.876753823489376</v>
       </c>
       <c r="K17" t="n">
-        <v>0.887996460681294</v>
+        <v>0.7103726111456587</v>
       </c>
     </row>
     <row r="18">
@@ -4868,31 +4868,31 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>132</v>
+        <v>271</v>
       </c>
       <c r="D18" t="n">
-        <v>2.866764171025353</v>
+        <v>12.84559291283292</v>
       </c>
       <c r="E18" t="n">
-        <v>4.366497925683041</v>
+        <v>19.75635822675999</v>
       </c>
       <c r="F18" t="n">
-        <v>7.737802122944278</v>
+        <v>26.61372465755518</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8448152264237136</v>
+        <v>-0.8172615919632893</v>
       </c>
       <c r="H18" t="n">
-        <v>31.86163441122522</v>
+        <v>11.32169312369476</v>
       </c>
       <c r="I18" t="n">
-        <v>12.23543353844474</v>
+        <v>12.22954181132504</v>
       </c>
       <c r="J18" t="n">
-        <v>19.00859413144825</v>
+        <v>22.41959472589807</v>
       </c>
       <c r="K18" t="n">
-        <v>0.8933878614097266</v>
+        <v>0.8509545491074079</v>
       </c>
     </row>
     <row r="19">
@@ -4907,31 +4907,31 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>69</v>
+        <v>208</v>
       </c>
       <c r="D19" t="n">
-        <v>4.081126789681326</v>
+        <v>13.84199780817706</v>
       </c>
       <c r="E19" t="n">
-        <v>1.311888584674097</v>
+        <v>4.323162675903657</v>
       </c>
       <c r="F19" t="n">
-        <v>2.05073072280375</v>
+        <v>5.73075663185077</v>
       </c>
       <c r="G19" t="n">
-        <v>0.8338299094592184</v>
+        <v>-0.3436234941615954</v>
       </c>
       <c r="H19" t="n">
-        <v>4.334639090003693</v>
+        <v>8.038243618227868</v>
       </c>
       <c r="I19" t="n">
-        <v>1.550395305534122</v>
+        <v>2.630714025191922</v>
       </c>
       <c r="J19" t="n">
-        <v>2.177137877910224</v>
+        <v>3.667494929248991</v>
       </c>
       <c r="K19" t="n">
-        <v>0.9110882419285601</v>
+        <v>0.7521078284119701</v>
       </c>
     </row>
   </sheetData>
@@ -4946,7 +4946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5037,7 +5037,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus1_actual_vs_benchmark_testing.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus1_actual_vs_benchmark_testing.png</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus2_actual_vs_benchmark_testing.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus2_actual_vs_benchmark_testing.png</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus4_actual_vs_benchmark_testing.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus4_actual_vs_benchmark_testing.png</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus5_actual_vs_benchmark_testing.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus5_actual_vs_benchmark_testing.png</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus6_actual_vs_benchmark_testing.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus6_actual_vs_benchmark_testing.png</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus7_actual_vs_benchmark_testing.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/agus7_actual_vs_benchmark_testing.png</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/all_plants_actual_vs_benchmark_testing.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_actual_testing_plots/all_plants_actual_vs_benchmark_testing.png</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_comparison/testing_mape_model_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_comparison/testing_mape_model_comparison.png</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5446,7 +5446,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>82.38</v>
+        <v>89.69</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/benchmark_comparison/testing_rmse_model_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/benchmark_comparison/testing_rmse_model_comparison.png</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5501,7 +5501,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>78.8</v>
+        <v>89.7</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_01_agus1_cleaned_profile.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_01_agus1_cleaned_profile.png</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_02_agus2_cleaned_profile.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_02_agus2_cleaned_profile.png</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_03_agus4_cleaned_profile.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_03_agus4_cleaned_profile.png</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5666,7 +5666,7 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>230.98</v>
+        <v>230.97</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_04_agus5_cleaned_profile.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_04_agus5_cleaned_profile.png</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_05_agus6_cleaned_profile.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_05_agus6_cleaned_profile.png</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5807,7 +5807,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_06_agus7_cleaned_profile.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/cleaned_profiles/figure_4_06_agus7_cleaned_profile.png</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/day_ahead_forecast/total_cascade_day_ahead_forecast_with_benchmarks.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/day_ahead_forecast/total_cascade_day_ahead_forecast_with_benchmarks.png</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>233.42</v>
+        <v>225.04</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -5917,7 +5917,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/error_analysis/rbfnn_actual_vs_predicted_scatter.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/error_analysis/rbfnn_actual_vs_predicted_scatter.png</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5941,7 +5941,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>358.82</v>
+        <v>360.88</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/error_analysis/rbfnn_residual_distribution.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/error_analysis/rbfnn_residual_distribution.png</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -5996,7 +5996,7 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>87.34999999999999</v>
+        <v>85.13</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -6027,7 +6027,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/error_analysis/rbfnn_testing_mape_per_plant.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/error_analysis/rbfnn_testing_mape_per_plant.png</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6051,7 +6051,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>61.61</v>
+        <v>60.57</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -6082,7 +6082,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/full_testing_split/agus1_testing_split_forecast_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/full_testing_split/agus1_testing_split_forecast_comparison.png</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/full_testing_split/agus2_testing_split_forecast_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/full_testing_split/agus2_testing_split_forecast_comparison.png</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/full_testing_split/agus4_testing_split_forecast_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/full_testing_split/agus4_testing_split_forecast_comparison.png</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6247,7 +6247,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/full_testing_split/agus5_testing_split_forecast_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/full_testing_split/agus5_testing_split_forecast_comparison.png</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/full_testing_split/agus6_testing_split_forecast_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/full_testing_split/agus6_testing_split_forecast_comparison.png</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/full_testing_split/agus7_testing_split_forecast_comparison.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/full_testing_split/agus7_testing_split_forecast_comparison.png</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6407,17 +6407,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>figure_4_13_agus1_testing_actual_vs_forecast.png</t>
+          <t>agus1_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_13_agus1_testing_actual_vs_forecast.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/testing/agus1_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>thesis_figures/testing_actual_vs_forecast/figure_4_13_agus1_testing_actual_vs_forecast.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/testing/agus1_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -6427,20 +6427,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>3570</t>
+          <t>2321</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1466</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>330.82</v>
+        <v>186.02</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>RBFNN testing actual versus forecast plot for Agus 1</t>
+          <t>Appendix testing or forecasting plot for Agus 1</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -6462,17 +6462,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>figure_4_14_agus2_testing_actual_vs_forecast.png</t>
+          <t>agus2_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_14_agus2_testing_actual_vs_forecast.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/testing/agus2_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>thesis_figures/testing_actual_vs_forecast/figure_4_14_agus2_testing_actual_vs_forecast.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/testing/agus2_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -6482,20 +6482,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3570</t>
+          <t>2321</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1466</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>246.79</v>
+        <v>151.97</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>RBFNN testing actual versus forecast plot for Agus 2</t>
+          <t>Appendix testing or forecasting plot for Agus 2</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -6517,17 +6517,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>figure_4_15_agus4_testing_actual_vs_forecast.png</t>
+          <t>agus4_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_15_agus4_testing_actual_vs_forecast.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/testing/agus4_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>thesis_figures/testing_actual_vs_forecast/figure_4_15_agus4_testing_actual_vs_forecast.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/testing/agus4_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -6537,20 +6537,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>3570</t>
+          <t>2321</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1466</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>247.14</v>
+        <v>147.2</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>RBFNN testing actual versus forecast plot for Agus 4</t>
+          <t>Appendix testing or forecasting plot for Agus 4</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -6572,17 +6572,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>figure_4_16_agus5_testing_actual_vs_forecast.png</t>
+          <t>agus5_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_16_agus5_testing_actual_vs_forecast.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/testing/agus5_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>thesis_figures/testing_actual_vs_forecast/figure_4_16_agus5_testing_actual_vs_forecast.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/testing/agus5_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -6592,20 +6592,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3570</t>
+          <t>2321</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1466</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>457.8</v>
+        <v>235.73</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>RBFNN testing actual versus forecast plot for Agus 5</t>
+          <t>Appendix testing or forecasting plot for Agus 5</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -6627,17 +6627,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>figure_4_17_agus6_testing_actual_vs_forecast.png</t>
+          <t>agus6_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_17_agus6_testing_actual_vs_forecast.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/testing/agus6_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>thesis_figures/testing_actual_vs_forecast/figure_4_17_agus6_testing_actual_vs_forecast.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/testing/agus6_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -6647,20 +6647,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>3570</t>
+          <t>2321</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1466</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>233.6</v>
+        <v>141.83</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>RBFNN testing actual versus forecast plot for Agus 6</t>
+          <t>Appendix testing or forecasting plot for Agus 6</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -6682,17 +6682,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>figure_4_18_agus7_testing_actual_vs_forecast.png</t>
+          <t>agus7_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_18_agus7_testing_actual_vs_forecast.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/testing/agus7_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>thesis_figures/testing_actual_vs_forecast/figure_4_18_agus7_testing_actual_vs_forecast.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/testing/agus7_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -6702,20 +6702,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>3570</t>
+          <t>2321</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1466</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>435.88</v>
+        <v>224.87</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>RBFNN testing actual versus forecast plot for Agus 7</t>
+          <t>Appendix testing or forecasting plot for Agus 7</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -6737,17 +6737,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>rbfnn_testing_mape_per_plant_maroon.png</t>
+          <t>all_plants_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/testing_metrics/rbfnn_testing_mape_per_plant_maroon.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/testing/all_plants_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>thesis_figures/testing_metrics/rbfnn_testing_mape_per_plant_maroon.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/testing/all_plants_testing_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -6757,20 +6757,20 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>2682</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>99.36</v>
+        <v>513.67</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>RBFNN testing metric plot</t>
+          <t>Appendix testing or forecasting plot for all Agus plants</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -6792,17 +6792,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>rbfnn_validation_mape_per_plant.png</t>
+          <t>agus1_validation_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>appendix_materials/figures/appendix_I_testing_plots/validation_metrics/rbfnn_validation_mape_per_plant.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/validation/agus1_validation_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>thesis_figures/validation_metrics/rbfnn_validation_mape_per_plant.png</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/validation/agus1_validation_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -6812,20 +6812,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>103.84</v>
+        <v>197.81</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>RBFNN validation metric plot</t>
+          <t>Appendix testing or forecasting plot for Agus 1</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -6842,22 +6842,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Appendix E</t>
+          <t>Appendix I</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>appendix_E_planned_outage_template.png</t>
+          <t>agus2_validation_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>appendix_materials/screenshots/appendix_E_planned_outage_template.png</t>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/validation/agus2_validation_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>outputs/outages_planning/Planned_Outages_Input.xlsx</t>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/validation/agus2_validation_actual_vs_rbfnn_forecast.png</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -6867,20 +6867,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>4599</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>846</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>130.99</v>
+        <v>151.21</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Screenshot-style table image of the 24-hour planned outage input template.</t>
+          <t>Appendix testing or forecasting plot for Agus 2</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -6897,55 +6897,1760 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>agus4_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/validation/agus4_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/validation/agus4_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>846</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>132.33</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 4</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>P036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>agus5_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/validation/agus5_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/validation/agus5_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>846</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>229.37</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 5</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>P037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>agus6_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/validation/agus6_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/validation/agus6_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>846</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>245.32</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 6</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>P038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>agus7_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/validation/agus7_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/validation/agus7_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>846</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>220.64</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 7</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>P039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>all_plants_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_actual_vs_forecast/validation/all_plants_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_actual_vs_forecast/validation/all_plants_validation_actual_vs_rbfnn_forecast.png</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2679</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>559.75</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for all Agus plants</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>P040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>agus1_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/testing/agus1_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/testing/agus1_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>191.11</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 1</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>P041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>agus2_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/testing/agus2_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/testing/agus2_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>145.29</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 2</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>P042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>agus4_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/testing/agus4_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/testing/agus4_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>143.12</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 4</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>P043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>agus5_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/testing/agus5_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/testing/agus5_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>238.68</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 5</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>P044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>agus6_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/testing/agus6_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/testing/agus6_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>135.52</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 6</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>P045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>agus7_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/testing/agus7_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/testing/agus7_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>230.17</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 7</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>P046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>all_plants_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/testing/all_plants_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/testing/all_plants_testing_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2700</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>498.96</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for all Agus plants</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>P047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>agus1_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/validation/agus1_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/validation/agus1_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>203.64</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 1</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>P048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>agus2_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/validation/agus2_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/validation/agus2_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>147.42</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 2</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>P049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>agus4_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/validation/agus4_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/validation/agus4_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>127.98</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 4</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>P050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>agus5_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/validation/agus5_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/validation/agus5_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>239.8</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 5</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>P051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>agus6_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/validation/agus6_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/validation/agus6_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>252.47</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 6</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>P052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>agus7_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/validation/agus7_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/validation/agus7_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>228.39</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for Agus 7</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>P053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>all_plants_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/rbfnn_outage_informed_actual_vs_forecast/validation/all_plants_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>thesis_figures/rbfnn_outage_informed_actual_vs_forecast/validation/all_plants_validation_actual_vs_rbfnn_outage_informed_forecast.png</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2700</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>562.73</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Appendix testing or forecasting plot for all Agus plants</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>P054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>figure_4_13_agus1_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_13_agus1_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>thesis_figures/testing_actual_vs_forecast/figure_4_13_agus1_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>3570</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>1466</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>336.96</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>RBFNN testing actual versus forecast plot for Agus 1</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>P055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>figure_4_14_agus2_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_14_agus2_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>thesis_figures/testing_actual_vs_forecast/figure_4_14_agus2_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>3570</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>1466</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>257.06</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>RBFNN testing actual versus forecast plot for Agus 2</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>P056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>figure_4_15_agus4_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_15_agus4_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>thesis_figures/testing_actual_vs_forecast/figure_4_15_agus4_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>3570</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>1466</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>251.77</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>RBFNN testing actual versus forecast plot for Agus 4</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>P057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>figure_4_16_agus5_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_16_agus5_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>thesis_figures/testing_actual_vs_forecast/figure_4_16_agus5_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>3570</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>1466</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>448.77</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>RBFNN testing actual versus forecast plot for Agus 5</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>P058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>figure_4_17_agus6_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_17_agus6_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>thesis_figures/testing_actual_vs_forecast/figure_4_17_agus6_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>3570</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>1466</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>237.25</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>RBFNN testing actual versus forecast plot for Agus 6</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>P059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>figure_4_18_agus7_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/testing_actual_vs_forecast/figure_4_18_agus7_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>thesis_figures/testing_actual_vs_forecast/figure_4_18_agus7_testing_actual_vs_forecast.png</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>3570</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>1466</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>431.4</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>RBFNN testing actual versus forecast plot for Agus 7</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>P060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>rbfnn_testing_mape_per_plant_maroon.png</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/testing_metrics/rbfnn_testing_mape_per_plant_maroon.png</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>thesis_figures/testing_metrics/rbfnn_testing_mape_per_plant_maroon.png</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>1860</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>99.36</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>RBFNN testing metric plot</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>P061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Appendix I</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>rbfnn_validation_mape_per_plant.png</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/appendix_I_testing_plots/validation_metrics/rbfnn_validation_mape_per_plant.png</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>thesis_figures/validation_metrics/rbfnn_validation_mape_per_plant.png</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>1860</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>103.84</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>RBFNN validation metric plot</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>P062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Appendix figure</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>thesis_code_block_diagram_clear.png</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/thesis_code_block_diagram_clear.png</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Generated inside appendix_materials</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2600</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>1750</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>298.47</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Appendix image file: thesis code block diagram clear.</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>P063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Appendix figure</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>thesis_code_block_diagram_neat.png</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/thesis_code_block_diagram_neat.png</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Generated inside appendix_materials</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>3300</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>322.36</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Appendix image file: thesis code block diagram neat.</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>P064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Appendix figure</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>thesis_code_block_diagram_portrait_top_to_bottom.png</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/figures/thesis_code_block_diagram_portrait_top_to_bottom.png</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Generated inside appendix_materials</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>3600</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>329.41</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Appendix image file: thesis code block diagram portrait top to bottom.</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>P065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Appendix E</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>appendix_E_planned_outage_template.png</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/screenshots/appendix_E_planned_outage_template.png</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>outputs/outages_planning/Planned_Outages_Input.xlsx</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>PNG image</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>4599</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>1872</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>130.99</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Screenshot-style table image of the 24-hour planned outage input template.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Use as an appendix figure or supporting visual reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>P066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
           <t>Appendix F</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>appendix_F_day_ahead_forecast_output.png</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>appendix_materials/screenshots/appendix_F_day_ahead_forecast_output.png</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>PAPER CONTEXT/screenshots/appendix_F_day_ahead_forecast_output.png</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>outputs/rbfnn_forecast/Day_Ahead_24H_RBFNN_Forecast.xlsx</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>PNG image</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>4662</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H67" t="inlineStr">
         <is>
           <t>1872</t>
         </is>
       </c>
-      <c r="I36" t="n">
-        <v>624.55</v>
-      </c>
-      <c r="J36" t="inlineStr">
+      <c r="I67" t="n">
+        <v>622.77</v>
+      </c>
+      <c r="J67" t="inlineStr">
         <is>
           <t>Screenshot-style table image of the 24-hour day-ahead RBFNN forecast output.</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K67" t="inlineStr">
         <is>
           <t>Use as an appendix figure or supporting visual reference.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K36"/>
+  <autoFilter ref="A1:K67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>